<commit_message>
Mise à jour de l'identifier type du rpps rang (INTRN --> RPPS) (#273)
* update identifier type pour rpps rang

* Update FRCoreOrganizationEtablissementProfile.fsh

* update translations

* add rpps rang identifier

* Update RPPS rang description in profile 08475511e35596437948074ff6260a7c4a497d44
</commit_message>
<xml_diff>
--- a/main/ig/CodeSystem-fr-core-cs-v2-0203.xlsx
+++ b/main/ig/CodeSystem-fr-core-cs-v2-0203.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="80">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-20T07:09:47+00:00</t>
+    <t>2026-03-25T10:22:11+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -126,7 +126,7 @@
     <t>Count</t>
   </si>
   <si>
-    <t>17</t>
+    <t>18</t>
   </si>
   <si>
     <t>Level</t>
@@ -154,6 +154,15 @@
   </si>
   <si>
     <t>N° RPPS</t>
+  </si>
+  <si>
+    <t>RPPSRG</t>
+  </si>
+  <si>
+    <t>N° RPPS Rang</t>
+  </si>
+  <si>
+    <t>N° RPPS Rang d'identification des cabinets libéraux selon le référentiel RPPS</t>
   </si>
   <si>
     <t>IDNPS</t>
@@ -561,7 +570,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -617,7 +626,7 @@
         <v>48</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5">
@@ -625,13 +634,13 @@
         <v>42</v>
       </c>
       <c r="B5" t="s" s="2">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C5" t="s" s="2">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6">
@@ -639,13 +648,13 @@
         <v>42</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C6" t="s" s="2">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D6" t="s" s="2">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7">
@@ -653,13 +662,13 @@
         <v>42</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C7" t="s" s="2">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D7" t="s" s="2">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8">
@@ -667,13 +676,13 @@
         <v>42</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C8" t="s" s="2">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D8" t="s" s="2">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9">
@@ -681,13 +690,13 @@
         <v>42</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C9" t="s" s="2">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D9" t="s" s="2">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10">
@@ -695,13 +704,13 @@
         <v>42</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C10" t="s" s="2">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D10" t="s" s="2">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11">
@@ -709,13 +718,13 @@
         <v>42</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C11" t="s" s="2">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D11" t="s" s="2">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12">
@@ -723,13 +732,13 @@
         <v>42</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C12" t="s" s="2">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D12" t="s" s="2">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="13">
@@ -737,13 +746,13 @@
         <v>42</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C13" t="s" s="2">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D13" t="s" s="2">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14">
@@ -751,13 +760,13 @@
         <v>42</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C14" t="s" s="2">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D14" t="s" s="2">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15">
@@ -765,13 +774,13 @@
         <v>42</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C15" t="s" s="2">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D15" t="s" s="2">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="16">
@@ -779,13 +788,13 @@
         <v>42</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C16" t="s" s="2">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D16" t="s" s="2">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17">
@@ -793,13 +802,13 @@
         <v>42</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C17" t="s" s="2">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D17" t="s" s="2">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="18">
@@ -807,13 +816,27 @@
         <v>42</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C18" t="s" s="2">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D18" t="s" s="2">
-        <v>76</v>
+        <v>77</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="2">
+        <v>42</v>
+      </c>
+      <c r="B19" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="C19" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="D19" t="s" s="2">
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>